<commit_message>
Added new column keeta in uploader sample
</commit_message>
<xml_diff>
--- a/public/uploadersSample/Items-Uploader-Sample.xlsx
+++ b/public/uploadersSample/Items-Uploader-Sample.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\HORIA DELIVERY\Horia-Delivery-Management-Website\backend\public\uploadersSample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{096690ED-5C6D-44FF-A3EC-DDCA370FBEFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{00D153DB-34B8-4A2C-A284-776A52459714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{626294E4-E408-4401-A983-15FCB8FB7A65}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{842387EB-878E-40F2-8B8C-E332A8037E92}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,14 +36,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+  <si>
+    <t>Falcon ID</t>
+  </si>
   <si>
     <t>Name</t>
   </si>
   <si>
-    <t>Falcon ID</t>
-  </si>
-  <si>
     <t>Driver/Rider</t>
   </si>
   <si>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t>Total</t>
+  </si>
+  <si>
+    <t>Keeta</t>
   </si>
 </sst>
 </file>
@@ -113,11 +116,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -451,33 +451,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC60B30C-F6C6-4C05-9DEF-7F5371BD8107}">
-  <dimension ref="A1:N1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87C2C009-483B-4460-B116-503232AF668E}">
+  <dimension ref="A1:O1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="4.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="9.140625" style="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -498,26 +481,29 @@
         <v>7</v>
       </c>
       <c r="I1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="VUpcwtVwopfk4XOF4zZh33m1CVLN1pSfm3c/HEIWHLXYUjk4h/lbNBsPBQ2qKq0ekWrx0QNzQLJyLXRTWqjstA==" saltValue="kmEl22C82k0V7lrPMjy3ag==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="YNoZciNWX3MIsZFx0CqBjY3Jdjv+qLM80ntAqF/Ycp2f7VnL7ulxS4Ryvkqa8GZlqoVus7lp9NqFQursOdQZAQ==" saltValue="tBhwb/us+lxCLrsbS1Fqng==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>